<commit_message>
POKEMONKEY 2.7: RAB RNR Excel, pratinjau & PDF seragam; uraian bisa diberi spasi
- Template RAB RNR: kotak persetujuan sisa HCGA (Dibuat/Diverifikasi/Pimpinan
  Site) dibuang, kotak Div Head bergaris, kolom Kode/Desc WBS/Uraian turun baris,
  kolom Kode WBS dilebarkan. Kotak Operation & HCA Director diberi garis saat
  total > Rp 25 juta (TemplatXlsx.salinGaya).
- Tinggi baris uraian dihitung dari lebar huruf Arial (tinggiBarisRab) dan
  dipakai sama oleh ekspor Excel dan pratinjau/PDF.
- Pratinjau: lebar kolom Minggu I–IV sama dengan Excel, kotak persetujuan
  bergaris penuh, sel minggu kosong tidak ditulis "Rp -".
- Tabel isian manual: spasi di akhir uraian tidak lagi terpangkas saat mengetik.
- Katalog: tombol sunting per uraian; katalog RAB tersedia di mode demo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/template-rab-rnr.xlsx
+++ b/public/template-rab-rnr.xlsx
@@ -857,7 +857,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="74">
+  <borders count="77">
     <border>
       <left/>
       <right/>
@@ -1784,6 +1784,41 @@
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -1793,7 +1828,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="214">
+  <cellXfs count="220">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2331,6 +2366,24 @@
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf applyBorder="1" numFmtId="0" fontId="6" fillId="0" borderId="73" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf applyBorder="1" numFmtId="0" fontId="6" fillId="0" borderId="74" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="75" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="76" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2466,1663 +2519,6 @@
             <a:solidFill>
               <a:sysClr val="windowText" lastClr="000000"/>
             </a:solidFill>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>15437</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>149453</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>931608</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>72004</xdr:rowOff>
-    </xdr:to>
-    <xdr:grpSp>
-      <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="1039" name="Group 1038">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30B68D3E-BDD1-A499-B466-1F512679299E}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvGrpSpPr/>
-      </xdr:nvGrpSpPr>
-      <xdr:grpSpPr>
-        <a:xfrm>
-          <a:off x="4542080" y="1637167"/>
-          <a:ext cx="7139171" cy="1455623"/>
-          <a:chOff x="9304579" y="1936524"/>
-          <a:chExt cx="7139171" cy="1301408"/>
-        </a:xfrm>
-      </xdr:grpSpPr>
-      <xdr:grpSp>
-        <xdr:nvGrpSpPr>
-          <xdr:cNvPr id="60" name="Group 59">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A1C5354E-AE9F-B187-4EF4-9442639F7C7E}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvGrpSpPr/>
-        </xdr:nvGrpSpPr>
-        <xdr:grpSpPr>
-          <a:xfrm>
-            <a:off x="9304579" y="1936524"/>
-            <a:ext cx="7139171" cy="1301408"/>
-            <a:chOff x="4933546" y="1699271"/>
-            <a:chExt cx="7128007" cy="1319551"/>
-          </a:xfrm>
-        </xdr:grpSpPr>
-        <xdr:grpSp>
-          <xdr:nvGrpSpPr>
-            <xdr:cNvPr id="56" name="Group 55">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{33FA1FB4-CA8E-FB4D-1247-AB5CA4AC0084}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGrpSpPr/>
-          </xdr:nvGrpSpPr>
-          <xdr:grpSpPr>
-            <a:xfrm>
-              <a:off x="4933546" y="1699271"/>
-              <a:ext cx="7125875" cy="1319551"/>
-              <a:chOff x="4938430" y="1704155"/>
-              <a:chExt cx="7125875" cy="1319551"/>
-            </a:xfrm>
-          </xdr:grpSpPr>
-          <xdr:cxnSp macro="">
-            <xdr:nvCxnSpPr>
-              <xdr:cNvPr id="35" name="Straight Connector 34">
-                <a:extLst>
-                  <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0E953AE-14A9-4474-BE73-FA10679F7CEF}"/>
-                  </a:ext>
-                </a:extLst>
-              </xdr:cNvPr>
-              <xdr:cNvCxnSpPr/>
-            </xdr:nvCxnSpPr>
-            <xdr:spPr>
-              <a:xfrm>
-                <a:off x="10296769" y="1738923"/>
-                <a:ext cx="0" cy="277028"/>
-              </a:xfrm>
-              <a:prstGeom prst="line">
-                <a:avLst/>
-              </a:prstGeom>
-              <a:ln w="9525">
-                <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000"/>
-                </a:solidFill>
-              </a:ln>
-            </xdr:spPr>
-            <xdr:style>
-              <a:lnRef idx="2">
-                <a:schemeClr val="accent1"/>
-              </a:lnRef>
-              <a:fillRef idx="0">
-                <a:schemeClr val="accent1"/>
-              </a:fillRef>
-              <a:effectRef idx="1">
-                <a:schemeClr val="accent1"/>
-              </a:effectRef>
-              <a:fontRef idx="minor">
-                <a:schemeClr val="tx1"/>
-              </a:fontRef>
-            </xdr:style>
-          </xdr:cxnSp>
-          <xdr:grpSp>
-            <xdr:nvGrpSpPr>
-              <xdr:cNvPr id="51" name="Group 50">
-                <a:extLst>
-                  <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3C171D4D-2AE5-9728-6A6D-8D4243DA3EF8}"/>
-                  </a:ext>
-                </a:extLst>
-              </xdr:cNvPr>
-              <xdr:cNvGrpSpPr/>
-            </xdr:nvGrpSpPr>
-            <xdr:grpSpPr>
-              <a:xfrm>
-                <a:off x="4938430" y="1704155"/>
-                <a:ext cx="7125875" cy="1319551"/>
-                <a:chOff x="4419963" y="1941407"/>
-                <a:chExt cx="7137039" cy="1301408"/>
-              </a:xfrm>
-            </xdr:grpSpPr>
-            <xdr:grpSp>
-              <xdr:nvGrpSpPr>
-                <xdr:cNvPr id="40" name="Group 39">
-                  <a:extLst>
-                    <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{73C24AB1-5B25-9663-12B4-DEDE86B2F00F}"/>
-                    </a:ext>
-                  </a:extLst>
-                </xdr:cNvPr>
-                <xdr:cNvGrpSpPr/>
-              </xdr:nvGrpSpPr>
-              <xdr:grpSpPr>
-                <a:xfrm>
-                  <a:off x="4419963" y="1941407"/>
-                  <a:ext cx="7137039" cy="1301408"/>
-                  <a:chOff x="8607332" y="1496904"/>
-                  <a:chExt cx="10270310" cy="1210694"/>
-                </a:xfrm>
-              </xdr:grpSpPr>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="4" name="Rectangle 3">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7564E30D-ADC3-FA74-2F10-9104B841A5D1}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="8607333" y="1537636"/>
-                    <a:ext cx="2575780" cy="1101817"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln w="9525"/>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="l"/>
-                    <a:endParaRPr lang="en-ID" sz="1100"/>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="5" name="Rectangle 4">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8A87A87D-1653-0989-A526-C694857572B7}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="11183114" y="1537636"/>
-                    <a:ext cx="2575780" cy="1101817"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln w="9525"/>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="l"/>
-                    <a:endParaRPr lang="en-ID" sz="1100"/>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="6" name="Rectangle 5">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AD8F23DD-C457-9BC6-F967-BD7573FB7D55}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="13758893" y="1720401"/>
-                    <a:ext cx="2569392" cy="919050"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln w="9525"/>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="l"/>
-                    <a:endParaRPr lang="en-ID" sz="1100"/>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="7" name="Rectangle 6">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{419786AD-37CC-1CC9-7B57-518AB67F504A}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="8607333" y="1537636"/>
-                    <a:ext cx="2575780" cy="182766"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln w="9525"/>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="l"/>
-                    <a:endParaRPr lang="en-ID" sz="1100"/>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="8" name="Rectangle 7">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{65694E51-DF16-144E-DCF4-C64EC030E6A0}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="11183114" y="1537636"/>
-                    <a:ext cx="2575780" cy="182766"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln w="9525"/>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="l"/>
-                    <a:endParaRPr lang="en-ID" sz="1100"/>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="9" name="Rectangle 8">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DF7FE455-311F-0581-8F26-C31E1E276787}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="13758893" y="1537636"/>
-                    <a:ext cx="5118749" cy="182766"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln w="9525"/>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="l"/>
-                    <a:endParaRPr lang="en-ID" sz="1100"/>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="10" name="Rectangle 9">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2DD2DCA3-C6C7-C4E0-E2D3-C4712F9FF7CA}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="8607332" y="2456685"/>
-                    <a:ext cx="2575780" cy="181721"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln w="9525"/>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="l"/>
-                    <a:endParaRPr lang="en-ID" sz="1100"/>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="11" name="Rectangle 10">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7636564C-0617-D6DB-D2F6-B255448721F9}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="9407274" y="1501083"/>
-                    <a:ext cx="975898" cy="287464"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="ctr"/>
-                    <a:r>
-                      <a:rPr lang="en-ID" sz="1100">
-                        <a:solidFill>
-                          <a:sysClr val="windowText" lastClr="000000"/>
-                        </a:solidFill>
-                      </a:rPr>
-                      <a:t>Dibuat Oleh,</a:t>
-                    </a:r>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="12" name="Rectangle 11">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6F1011CD-2617-3326-AFFA-2CD582F0BA53}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="11762956" y="1502127"/>
-                    <a:ext cx="1430669" cy="287464"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="ctr"/>
-                    <a:r>
-                      <a:rPr lang="en-ID" sz="1100">
-                        <a:solidFill>
-                          <a:sysClr val="windowText" lastClr="000000"/>
-                        </a:solidFill>
-                      </a:rPr>
-                      <a:t>Diverifikasi Oleh,</a:t>
-                    </a:r>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="13" name="Rectangle 12">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{8A99CA47-AA87-A8DB-48D8-4124E9396373}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="14351172" y="1496904"/>
-                    <a:ext cx="1753011" cy="249164"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:r>
-                      <a:rPr lang="en-ID" sz="1100">
-                        <a:solidFill>
-                          <a:sysClr val="windowText" lastClr="000000"/>
-                        </a:solidFill>
-                        <a:effectLst/>
-                        <a:latin typeface="+mn-lt"/>
-                        <a:ea typeface="+mn-ea"/>
-                        <a:cs typeface="+mn-cs"/>
-                      </a:rPr>
-                      <a:t>Disetujui Oleh,</a:t>
-                    </a:r>
-                    <a:endParaRPr lang="en-ID">
-                      <a:solidFill>
-                        <a:sysClr val="windowText" lastClr="000000"/>
-                      </a:solidFill>
-                      <a:effectLst/>
-                    </a:endParaRPr>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="14" name="Rectangle 13">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{398C4427-E096-C600-BE6A-A2A511536D63}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="11185730" y="2456686"/>
-                    <a:ext cx="2575780" cy="181721"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln w="9525"/>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="l"/>
-                    <a:endParaRPr lang="en-ID" sz="1100"/>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="15" name="Rectangle 14">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{539E023C-045B-484C-29C0-F81CCAB978D8}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="13761509" y="2456686"/>
-                    <a:ext cx="2566776" cy="181721"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln w="9525"/>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="l"/>
-                    <a:endParaRPr lang="en-ID" sz="1100"/>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="16" name="Rectangle 15">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9B13FC45-FEB5-D000-177D-9168EEA66EC3}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="16328287" y="2456686"/>
-                    <a:ext cx="2549355" cy="181721"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln w="9525"/>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="l"/>
-                    <a:endParaRPr lang="en-ID" sz="1100"/>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="17" name="Rectangle 16">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{11296174-607F-1AC4-1C07-E130D883DDD4}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="9041394" y="2252511"/>
-                    <a:ext cx="1739969" cy="214916"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="ctr"/>
-                    <a:r>
-                      <a:rPr lang="en-ID" sz="1100">
-                        <a:solidFill>
-                          <a:sysClr val="windowText" lastClr="000000"/>
-                        </a:solidFill>
-                      </a:rPr>
-                      <a:t>M. Yusriani</a:t>
-                    </a:r>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="19" name="Rectangle 18">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F6E803B8-DA5E-BDA7-1610-55503E957C4F}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="13764461" y="2243675"/>
-                    <a:ext cx="2535532" cy="236596"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="ctr"/>
-                    <a:r>
-                      <a:rPr lang="en-ID" sz="1100">
-                        <a:solidFill>
-                          <a:sysClr val="windowText" lastClr="000000"/>
-                        </a:solidFill>
-                        <a:effectLst/>
-                        <a:latin typeface="+mn-lt"/>
-                        <a:ea typeface="+mn-ea"/>
-                        <a:cs typeface="+mn-cs"/>
-                      </a:rPr>
-                      <a:t>Bambang</a:t>
-                    </a:r>
-                    <a:r>
-                      <a:rPr lang="en-ID" sz="1100" baseline="0">
-                        <a:solidFill>
-                          <a:sysClr val="windowText" lastClr="000000"/>
-                        </a:solidFill>
-                        <a:effectLst/>
-                        <a:latin typeface="+mn-lt"/>
-                        <a:ea typeface="+mn-ea"/>
-                        <a:cs typeface="+mn-cs"/>
-                      </a:rPr>
-                      <a:t> Octaryono</a:t>
-                    </a:r>
-                    <a:endParaRPr lang="en-ID">
-                      <a:solidFill>
-                        <a:sysClr val="windowText" lastClr="000000"/>
-                      </a:solidFill>
-                      <a:effectLst/>
-                    </a:endParaRPr>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="20" name="Rectangle 19">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3BBD76A2-EF8D-C1FB-A411-45E71F033C75}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="16555531" y="2260082"/>
-                    <a:ext cx="2191567" cy="257842"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="ctr"/>
-                    <a:r>
-                      <a:rPr lang="en-ID" sz="1100">
-                        <a:solidFill>
-                          <a:sysClr val="windowText" lastClr="000000"/>
-                        </a:solidFill>
-                      </a:rPr>
-                      <a:t>Cecep H. Setiadi</a:t>
-                    </a:r>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="21" name="Rectangle 20">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{46126565-DED3-8243-C804-590D9538CB48}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="9238865" y="1666355"/>
-                    <a:ext cx="1312716" cy="289814"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="ctr"/>
-                    <a:endParaRPr lang="en-ID" sz="1100">
-                      <a:solidFill>
-                        <a:sysClr val="windowText" lastClr="000000"/>
-                      </a:solidFill>
-                    </a:endParaRPr>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="22" name="Rectangle 21">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E3199677-58DC-0DF3-130C-F593EDA74987}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="11544323" y="1691673"/>
-                    <a:ext cx="1936021" cy="299129"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="ctr"/>
-                    <a:r>
-                      <a:rPr lang="en-ID" sz="1100">
-                        <a:solidFill>
-                          <a:sysClr val="windowText" lastClr="000000"/>
-                        </a:solidFill>
-                      </a:rPr>
-                      <a:t>Finance</a:t>
-                    </a:r>
-                    <a:r>
-                      <a:rPr lang="en-ID" sz="1100" baseline="0">
-                        <a:solidFill>
-                          <a:sysClr val="windowText" lastClr="000000"/>
-                        </a:solidFill>
-                      </a:rPr>
-                      <a:t> Site</a:t>
-                    </a:r>
-                    <a:endParaRPr lang="en-ID" sz="1100">
-                      <a:solidFill>
-                        <a:sysClr val="windowText" lastClr="000000"/>
-                      </a:solidFill>
-                    </a:endParaRPr>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="23" name="Rectangle 22">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{97B11845-13A2-3487-8C66-4DAC78EFCBE4}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="14273120" y="1666355"/>
-                    <a:ext cx="1540066" cy="289814"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="ctr"/>
-                    <a:r>
-                      <a:rPr lang="en-ID" sz="1100" baseline="0">
-                        <a:solidFill>
-                          <a:sysClr val="windowText" lastClr="000000"/>
-                        </a:solidFill>
-                      </a:rPr>
-                      <a:t>Pimpinan Site</a:t>
-                    </a:r>
-                    <a:endParaRPr lang="en-ID" sz="1100">
-                      <a:solidFill>
-                        <a:sysClr val="windowText" lastClr="000000"/>
-                      </a:solidFill>
-                    </a:endParaRPr>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="24" name="Rectangle 23">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EA7B00B7-AA65-BEB5-7154-638A0996E269}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="16649304" y="1683234"/>
-                    <a:ext cx="1935127" cy="316007"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="ctr"/>
-                    <a:r>
-                      <a:rPr lang="en-ID" sz="1100">
-                        <a:solidFill>
-                          <a:sysClr val="windowText" lastClr="000000"/>
-                        </a:solidFill>
-                      </a:rPr>
-                      <a:t>Eng</a:t>
-                    </a:r>
-                    <a:r>
-                      <a:rPr lang="en-ID" sz="1100" baseline="0">
-                        <a:solidFill>
-                          <a:sysClr val="windowText" lastClr="000000"/>
-                        </a:solidFill>
-                      </a:rPr>
-                      <a:t> &amp; Opr. Div Head</a:t>
-                    </a:r>
-                    <a:endParaRPr lang="en-ID" sz="1100">
-                      <a:solidFill>
-                        <a:sysClr val="windowText" lastClr="000000"/>
-                      </a:solidFill>
-                    </a:endParaRPr>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="26" name="Rectangle 25">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2D7E6681-BBC9-73C1-E45C-3C7A7399814B}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="11132591" y="2412561"/>
-                    <a:ext cx="1312716" cy="287465"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="l"/>
-                    <a:r>
-                      <a:rPr lang="en-ID" sz="1100">
-                        <a:solidFill>
-                          <a:sysClr val="windowText" lastClr="000000"/>
-                        </a:solidFill>
-                      </a:rPr>
-                      <a:t>Tanggal :</a:t>
-                    </a:r>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="27" name="Rectangle 26">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{219FEF1B-4E2A-359F-9052-E3273F595BA5}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="13699950" y="2420133"/>
-                    <a:ext cx="2201640" cy="287465"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="l"/>
-                    <a:r>
-                      <a:rPr lang="en-ID" sz="1100">
-                        <a:solidFill>
-                          <a:sysClr val="windowText" lastClr="000000"/>
-                        </a:solidFill>
-                      </a:rPr>
-                      <a:t>Tanggal : </a:t>
-                    </a:r>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-              <xdr:sp macro="" textlink="">
-                <xdr:nvSpPr>
-                  <xdr:cNvPr id="28" name="Rectangle 27">
-                    <a:extLst>
-                      <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                        <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F083B597-653D-4C59-B7C9-F8CB483F9482}"/>
-                      </a:ext>
-                    </a:extLst>
-                  </xdr:cNvPr>
-                  <xdr:cNvSpPr/>
-                </xdr:nvSpPr>
-                <xdr:spPr>
-                  <a:xfrm>
-                    <a:off x="16249597" y="2412561"/>
-                    <a:ext cx="1312716" cy="287465"/>
-                  </a:xfrm>
-                  <a:prstGeom prst="rect">
-                    <a:avLst/>
-                  </a:prstGeom>
-                  <a:noFill/>
-                  <a:ln>
-                    <a:noFill/>
-                  </a:ln>
-                </xdr:spPr>
-                <xdr:style>
-                  <a:lnRef idx="2">
-                    <a:schemeClr val="accent1">
-                      <a:shade val="15000"/>
-                    </a:schemeClr>
-                  </a:lnRef>
-                  <a:fillRef idx="1">
-                    <a:schemeClr val="accent1"/>
-                  </a:fillRef>
-                  <a:effectRef idx="0">
-                    <a:schemeClr val="accent1"/>
-                  </a:effectRef>
-                  <a:fontRef idx="minor">
-                    <a:schemeClr val="lt1"/>
-                  </a:fontRef>
-                </xdr:style>
-                <xdr:txBody>
-                  <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                  <a:lstStyle/>
-                  <a:p>
-                    <a:pPr algn="l"/>
-                    <a:r>
-                      <a:rPr lang="en-ID" sz="1100">
-                        <a:solidFill>
-                          <a:sysClr val="windowText" lastClr="000000"/>
-                        </a:solidFill>
-                      </a:rPr>
-                      <a:t>Tanggal :</a:t>
-                    </a:r>
-                  </a:p>
-                </xdr:txBody>
-              </xdr:sp>
-            </xdr:grpSp>
-            <xdr:sp macro="" textlink="">
-              <xdr:nvSpPr>
-                <xdr:cNvPr id="36" name="Rectangle 35">
-                  <a:extLst>
-                    <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                      <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{71ED4DC6-652A-41FA-A6F4-111D2B42E097}"/>
-                    </a:ext>
-                  </a:extLst>
-                </xdr:cNvPr>
-                <xdr:cNvSpPr/>
-              </xdr:nvSpPr>
-              <xdr:spPr>
-                <a:xfrm>
-                  <a:off x="9779000" y="1948542"/>
-                  <a:ext cx="1750785" cy="292101"/>
-                </a:xfrm>
-                <a:prstGeom prst="rect">
-                  <a:avLst/>
-                </a:prstGeom>
-                <a:noFill/>
-                <a:ln>
-                  <a:noFill/>
-                </a:ln>
-              </xdr:spPr>
-              <xdr:style>
-                <a:lnRef idx="2">
-                  <a:schemeClr val="accent1">
-                    <a:shade val="15000"/>
-                  </a:schemeClr>
-                </a:lnRef>
-                <a:fillRef idx="1">
-                  <a:schemeClr val="accent1"/>
-                </a:fillRef>
-                <a:effectRef idx="0">
-                  <a:schemeClr val="accent1"/>
-                </a:effectRef>
-                <a:fontRef idx="minor">
-                  <a:schemeClr val="lt1"/>
-                </a:fontRef>
-              </xdr:style>
-              <xdr:txBody>
-                <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-                <a:lstStyle/>
-                <a:p>
-                  <a:pPr algn="ctr"/>
-                  <a:r>
-                    <a:rPr lang="en-ID" sz="1100">
-                      <a:solidFill>
-                        <a:sysClr val="windowText" lastClr="000000"/>
-                      </a:solidFill>
-                    </a:rPr>
-                    <a:t>Disetujui Oleh,</a:t>
-                  </a:r>
-                </a:p>
-              </xdr:txBody>
-            </xdr:sp>
-          </xdr:grpSp>
-        </xdr:grpSp>
-        <xdr:cxnSp macro="">
-          <xdr:nvCxnSpPr>
-            <xdr:cNvPr id="58" name="Straight Connector 57">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6128AF2A-2180-917B-31CB-6DB65CBA14E9}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvCxnSpPr/>
-          </xdr:nvCxnSpPr>
-          <xdr:spPr>
-            <a:xfrm flipH="1">
-              <a:off x="12054536" y="1937630"/>
-              <a:ext cx="7017" cy="901865"/>
-            </a:xfrm>
-            <a:prstGeom prst="line">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:ln w="9525">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
-            </a:ln>
-          </xdr:spPr>
-          <xdr:style>
-            <a:lnRef idx="2">
-              <a:schemeClr val="accent1"/>
-            </a:lnRef>
-            <a:fillRef idx="0">
-              <a:schemeClr val="accent1"/>
-            </a:fillRef>
-            <a:effectRef idx="1">
-              <a:schemeClr val="accent1"/>
-            </a:effectRef>
-            <a:fontRef idx="minor">
-              <a:schemeClr val="tx1"/>
-            </a:fontRef>
-          </xdr:style>
-        </xdr:cxnSp>
-      </xdr:grpSp>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="1037" name="Rectangle 1036">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9D03C463-6770-4242-BF78-D5B83793EFC1}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr/>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="9524999" y="2149927"/>
-            <a:ext cx="1345378" cy="321542"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:style>
-          <a:lnRef idx="2">
-            <a:schemeClr val="accent1">
-              <a:shade val="15000"/>
-            </a:schemeClr>
-          </a:lnRef>
-          <a:fillRef idx="1">
-            <a:schemeClr val="accent1"/>
-          </a:fillRef>
-          <a:effectRef idx="0">
-            <a:schemeClr val="accent1"/>
-          </a:effectRef>
-          <a:fontRef idx="minor">
-            <a:schemeClr val="lt1"/>
-          </a:fontRef>
-        </xdr:style>
-        <xdr:txBody>
-          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr algn="ctr"/>
-            <a:r>
-              <a:rPr lang="en-ID" sz="1050">
-                <a:solidFill>
-                  <a:sysClr val="windowText" lastClr="000000"/>
-                </a:solidFill>
-              </a:rPr>
-              <a:t>HCA Sect. Head</a:t>
-            </a:r>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-    </xdr:grpSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>1823357</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>326572</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>1308419</xdr:colOff>
-      <xdr:row>14</xdr:row>
-      <xdr:rowOff>3246</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="1047" name="Rectangle 1046">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1847D8F4-D788-4806-865A-D92135B165CA}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="6350000" y="2549072"/>
-          <a:ext cx="1761990" cy="284460"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="15000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-ID" sz="1100">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>Azmi</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ID" sz="1100" baseline="0">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t> Rahmadi &amp; M. Yusriani</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-ID">
-            <a:solidFill>
-              <a:sysClr val="windowText" lastClr="000000"/>
-            </a:solidFill>
-            <a:effectLst/>
           </a:endParaRPr>
         </a:p>
       </xdr:txBody>
@@ -4457,7 +2853,7 @@
   <cols>
     <col min="1" max="1" width="8.81640625" customWidth="1"/>
     <col min="2" max="2" width="4.54296875" customWidth="1"/>
-    <col min="3" max="3" width="17.54296875" customWidth="1"/>
+    <col min="3" max="3" width="19.26953125" customWidth="1"/>
     <col min="4" max="4" width="33.90625" customWidth="1"/>
     <col min="5" max="5" width="32.54296875" customWidth="1"/>
     <col min="6" max="9" width="18.81640625" customWidth="1"/>
@@ -4595,10 +2991,10 @@
         <v>4</v>
       </c>
       <c r="E10" s="88"/>
-      <c r="F10" s="175"/>
-      <c r="G10" s="175"/>
-      <c r="H10" s="176"/>
-      <c r="I10" s="177"/>
+      <c r="F10" s="177"/>
+      <c r="G10" s="176"/>
+      <c r="H10" s="175"/>
+      <c r="I10" s="175"/>
       <c r="J10" s="111"/>
       <c r="K10" s="7"/>
       <c r="N10" s="120" t="s">
@@ -4613,8 +3009,8 @@
       <c r="C11" s="99"/>
       <c r="D11" s="114"/>
       <c r="E11" s="7"/>
-      <c r="F11" s="148"/>
-      <c r="G11" s="148"/>
+      <c r="F11" s="216"/>
+      <c r="G11" s="217"/>
       <c r="H11" s="148"/>
       <c r="I11" s="148"/>
       <c r="J11" s="89"/>
@@ -4631,8 +3027,8 @@
       <c r="C12" s="101"/>
       <c r="D12" s="149"/>
       <c r="E12" s="148"/>
-      <c r="F12" s="148"/>
-      <c r="G12" s="148"/>
+      <c r="F12" s="216"/>
+      <c r="G12" s="217"/>
       <c r="H12" s="148"/>
       <c r="I12" s="148"/>
       <c r="J12" s="151"/>
@@ -4644,8 +3040,8 @@
       <c r="C13" s="103"/>
       <c r="D13" s="150"/>
       <c r="E13" s="148"/>
-      <c r="F13" s="148"/>
-      <c r="G13" s="148"/>
+      <c r="F13" s="216"/>
+      <c r="G13" s="217"/>
       <c r="H13" s="148"/>
       <c r="I13" s="148"/>
       <c r="J13" s="151"/>
@@ -4659,8 +3055,8 @@
       <c r="C14" s="4"/>
       <c r="D14" s="115"/>
       <c r="E14" s="148"/>
-      <c r="F14" s="148"/>
-      <c r="G14" s="148"/>
+      <c r="F14" s="216"/>
+      <c r="G14" s="217"/>
       <c r="H14" s="148"/>
       <c r="I14" s="148"/>
       <c r="J14" s="151"/>
@@ -4674,10 +3070,10 @@
       <c r="C15" s="91"/>
       <c r="D15" s="116"/>
       <c r="E15" s="90"/>
-      <c r="F15" s="139"/>
-      <c r="G15" s="139"/>
-      <c r="H15" s="140"/>
-      <c r="I15" s="141"/>
+      <c r="F15" s="218"/>
+      <c r="G15" s="219"/>
+      <c r="H15" s="139"/>
+      <c r="I15" s="139"/>
       <c r="J15" s="112"/>
       <c r="K15" s="8"/>
       <c r="N15" s="123" t="s">
@@ -4742,12 +3138,9 @@
       <c r="B19" s="10">
         <v>1</v>
       </c>
-      <c r="C19" s="14"/>
-      <c r="D19" t="e">
-        <f>VLOOKUP(C19,WBS!$B:$C,2,0)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="E19" s="11" t="s">
+      <c r="C19" s="214"/>
+      <c r="D19" s="214"/>
+      <c r="E19" s="215" t="s">
         <v>14</v>
       </c>
       <c r="F19" s="92">
@@ -4777,9 +3170,9 @@
         <f>1+B19</f>
         <v>2</v>
       </c>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14" t="s">
+      <c r="C20" s="214"/>
+      <c r="D20" s="214"/>
+      <c r="E20" s="214" t="s">
         <v>15</v>
       </c>
       <c r="F20" s="93">
@@ -4809,9 +3202,9 @@
         <f>1+B20</f>
         <v>3</v>
       </c>
-      <c r="C21" s="14"/>
-      <c r="D21" s="14"/>
-      <c r="E21" s="14" t="s">
+      <c r="C21" s="214"/>
+      <c r="D21" s="214"/>
+      <c r="E21" s="214" t="s">
         <v>16</v>
       </c>
       <c r="F21" s="93">
@@ -4841,9 +3234,9 @@
         <f>1+B21</f>
         <v>4</v>
       </c>
-      <c r="C22" s="14"/>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14" t="s">
+      <c r="C22" s="214"/>
+      <c r="D22" s="214"/>
+      <c r="E22" s="214" t="s">
         <v>191</v>
       </c>
       <c r="F22" s="94">
@@ -4874,9 +3267,9 @@
         <f>1+B22</f>
         <v>5</v>
       </c>
-      <c r="C23" s="14"/>
-      <c r="D23" s="14"/>
-      <c r="E23" s="15" t="s">
+      <c r="C23" s="214"/>
+      <c r="D23" s="214"/>
+      <c r="E23" s="214" t="s">
         <v>17</v>
       </c>
       <c r="F23" s="94">
@@ -4906,9 +3299,9 @@
         <f>1+B23</f>
         <v>6</v>
       </c>
-      <c r="C24" s="14"/>
-      <c r="D24" s="14"/>
-      <c r="E24" s="15" t="s">
+      <c r="C24" s="214"/>
+      <c r="D24" s="214"/>
+      <c r="E24" s="214" t="s">
         <v>79</v>
       </c>
       <c r="F24" s="94">
@@ -4938,9 +3331,9 @@
         <f>1+B24</f>
         <v>7</v>
       </c>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-      <c r="E25" s="15" t="s">
+      <c r="C25" s="214"/>
+      <c r="D25" s="214"/>
+      <c r="E25" s="214" t="s">
         <v>80</v>
       </c>
       <c r="F25" s="94">
@@ -4970,9 +3363,9 @@
         <f>1+B25</f>
         <v>8</v>
       </c>
-      <c r="C26" s="14"/>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14" t="s">
+      <c r="C26" s="214"/>
+      <c r="D26" s="214"/>
+      <c r="E26" s="214" t="s">
         <v>18</v>
       </c>
       <c r="F26" s="94">
@@ -5002,9 +3395,9 @@
         <f>1+B26</f>
         <v>9</v>
       </c>
-      <c r="C27" s="16"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="17" t="s">
+      <c r="C27" s="214"/>
+      <c r="D27" s="214"/>
+      <c r="E27" s="214" t="s">
         <v>19</v>
       </c>
       <c r="F27" s="94">
@@ -5034,9 +3427,9 @@
         <f>1+B27</f>
         <v>10</v>
       </c>
-      <c r="C28" s="16"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="18" t="s">
+      <c r="C28" s="214"/>
+      <c r="D28" s="214"/>
+      <c r="E28" s="214" t="s">
         <v>81</v>
       </c>
       <c r="F28" s="94"/>
@@ -5054,9 +3447,9 @@
         <f>1+B28</f>
         <v>11</v>
       </c>
-      <c r="C29" s="16"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="18"/>
+      <c r="C29" s="214"/>
+      <c r="D29" s="214"/>
+      <c r="E29" s="214"/>
       <c r="F29" s="94"/>
       <c r="G29" s="95"/>
       <c r="H29" s="95"/>
@@ -5072,9 +3465,9 @@
         <f>1+B29</f>
         <v>12</v>
       </c>
-      <c r="C30" s="16"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="18" t="s">
+      <c r="C30" s="214"/>
+      <c r="D30" s="214"/>
+      <c r="E30" s="214" t="s">
         <v>82</v>
       </c>
       <c r="F30" s="94"/>
@@ -5092,9 +3485,9 @@
         <f>1+B30</f>
         <v>13</v>
       </c>
-      <c r="C31" s="16"/>
-      <c r="D31" s="16"/>
-      <c r="E31" s="18" t="s">
+      <c r="C31" s="214"/>
+      <c r="D31" s="214"/>
+      <c r="E31" s="214" t="s">
         <v>82</v>
       </c>
       <c r="F31" s="94"/>
@@ -5112,9 +3505,9 @@
         <f>1+B31</f>
         <v>14</v>
       </c>
-      <c r="C32" s="16"/>
-      <c r="D32" s="16"/>
-      <c r="E32" s="18" t="s">
+      <c r="C32" s="214"/>
+      <c r="D32" s="214"/>
+      <c r="E32" s="214" t="s">
         <v>82</v>
       </c>
       <c r="F32" s="95"/>

</xml_diff>

<commit_message>
POKEMONKEY 2.11: RAB RNR per kategori dengan lembar Excel tersambung; Memo gaya Notion
RAB RNR
- Tiap uraian boleh diberi kategori (ATK, BBM, Catering, Perdin & Cuti,
  Listrik PLN, Air PDAM, Telp & Internet, Pantry, KHL); kategori ikut dari
  katalog saat ADD, bisa diubah di kartu papan, tabel manual, dan Kelola katalog.
- Ekspor Excel: lembar rekap tetap satu baris per uraian; nilai minggu uraian
  berkategori merujuk lembar rincian W1-W4 kategorinya (format template RAB
  HCGA). Uraian tanpa kategori tetap ditulis langsung di rekap.
- Template RAB RNR mendapat lembar model "Kategori"; xlsx-templat bisa membuka,
  menggandakan, dan menghapus lembar.
- Katalog server mengirim dan menyimpan kategori.

Memo gaya Notion (migrasi 0027): editor blok, properti, tugas, kalender,
bagikan lewat tautan.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/template-rab-rnr.xlsx
+++ b/public/template-rab-rnr.xlsx
@@ -14,9 +14,11 @@
   </bookViews>
   <sheets>
     <sheet name="RAB RNR" sheetId="1" r:id="rId2"/>
+    <sheet name="Kategori" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'RAB RNR'!$B$2:$J$34</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">Kategori!$B$2:$H$67</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <fileRecoveryPr repairLoad="1"/>
@@ -2523,6 +2525,61 @@
         </a:p>
       </xdr:txBody>
     </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>78106</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>157564</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>426720</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>160136</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{356111A9-ED9D-4728-8CB8-FB8DB40226F9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1144906" y="157564"/>
+          <a:ext cx="706754" cy="703612"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -3605,6 +3662,641 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{85DC5CF2-EBEC-4C94-9F75-EB19607A1B9E}">
+  <sheetPr codeName="Sheet9">
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="C2:H67"/>
+  <sheetFormatPr defaultColWidth="9.26953125" defaultRowHeight="13"/>
+  <cols>
+    <col min="1" max="2" width="7.7265625" style="20" customWidth="1"/>
+    <col min="3" max="3" width="5.26953125" style="20" customWidth="1"/>
+    <col min="4" max="4" width="41.7265625" style="20" customWidth="1"/>
+    <col min="5" max="5" width="11.453125" style="20" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.54296875" style="20" customWidth="1"/>
+    <col min="7" max="7" width="20.26953125" style="20" customWidth="1"/>
+    <col min="8" max="8" width="16.7265625" style="20" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="1.453125" style="20" customWidth="1"/>
+    <col min="10" max="10" width="9.26953125" style="20"/>
+    <col min="11" max="11" width="11.7265625" style="20" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.26953125" style="20"/>
+  </cols>
+  <sheetData>
+    <row r="2">
+      <c r="C2" s="195" t="s">
+        <v>74</v>
+      </c>
+      <c r="D2" s="196"/>
+      <c r="E2" s="196"/>
+      <c r="F2" s="196"/>
+      <c r="G2" s="196"/>
+      <c r="H2" s="196"/>
+    </row>
+    <row r="3">
+      <c r="C3" s="196"/>
+      <c r="D3" s="196"/>
+      <c r="E3" s="196"/>
+      <c r="F3" s="196"/>
+      <c r="G3" s="196"/>
+      <c r="H3" s="196"/>
+    </row>
+    <row r="4">
+      <c r="C4" s="196"/>
+      <c r="D4" s="196"/>
+      <c r="E4" s="196"/>
+      <c r="F4" s="196"/>
+      <c r="G4" s="196"/>
+      <c r="H4" s="196"/>
+    </row>
+    <row r="5">
+      <c r="C5" s="196"/>
+      <c r="D5" s="196"/>
+      <c r="E5" s="196"/>
+      <c r="F5" s="196"/>
+      <c r="G5" s="196"/>
+      <c r="H5" s="196"/>
+    </row>
+    <row r="6" ht="13.5" thickBot="1"/>
+    <row r="7" ht="18" customHeight="1" thickBot="1">
+      <c r="C7" s="186"/>
+      <c r="D7" s="187"/>
+      <c r="E7" s="187"/>
+      <c r="F7" s="187"/>
+      <c r="G7" s="187"/>
+      <c r="H7" s="188"/>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="C8" s="189" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="191" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="191" t="s">
+        <v>22</v>
+      </c>
+      <c r="F8" s="191" t="s">
+        <v>23</v>
+      </c>
+      <c r="G8" s="191" t="s">
+        <v>24</v>
+      </c>
+      <c r="H8" s="193" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" ht="13.9" customHeight="1" thickBot="1">
+      <c r="C9" s="190"/>
+      <c r="D9" s="192"/>
+      <c r="E9" s="192"/>
+      <c r="F9" s="192"/>
+      <c r="G9" s="192"/>
+      <c r="H9" s="194"/>
+    </row>
+    <row r="10" ht="14.5" customHeight="1">
+      <c r="C10" s="21"/>
+      <c r="D10" s="27"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="23"/>
+      <c r="G10" s="28"/>
+      <c r="H10" s="25"/>
+    </row>
+    <row r="11" ht="14.5" customHeight="1">
+      <c r="C11" s="21"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="23"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="25"/>
+    </row>
+    <row r="12" ht="14.5" customHeight="1">
+      <c r="C12" s="21"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="28"/>
+      <c r="H12" s="25"/>
+    </row>
+    <row r="13" ht="14.5" customHeight="1">
+      <c r="C13" s="21"/>
+      <c r="D13" s="27"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="23"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="25"/>
+    </row>
+    <row r="14" ht="14.5" customHeight="1">
+      <c r="C14" s="21"/>
+      <c r="D14" s="27"/>
+      <c r="E14" s="23"/>
+      <c r="F14" s="23"/>
+      <c r="G14" s="28"/>
+      <c r="H14" s="25"/>
+    </row>
+    <row r="15" ht="14.5" customHeight="1">
+      <c r="C15" s="21"/>
+      <c r="D15" s="27"/>
+      <c r="E15" s="23"/>
+      <c r="F15" s="23"/>
+      <c r="G15" s="28"/>
+      <c r="H15" s="25"/>
+    </row>
+    <row r="16" ht="14.5" customHeight="1">
+      <c r="C16" s="21"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="23"/>
+      <c r="F16" s="23"/>
+      <c r="G16" s="28"/>
+      <c r="H16" s="25"/>
+    </row>
+    <row r="17" ht="14.5" customHeight="1">
+      <c r="C17" s="21"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="23"/>
+      <c r="F17" s="23"/>
+      <c r="G17" s="28"/>
+      <c r="H17" s="25"/>
+    </row>
+    <row r="18" ht="14.5" customHeight="1">
+      <c r="C18" s="21"/>
+      <c r="D18" s="27"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="23"/>
+      <c r="G18" s="28"/>
+      <c r="H18" s="25"/>
+    </row>
+    <row r="19" ht="15" thickBot="1">
+      <c r="C19" s="34"/>
+      <c r="D19" s="35"/>
+      <c r="E19" s="36"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="38"/>
+      <c r="H19" s="39"/>
+    </row>
+    <row r="20" ht="16.5" thickBot="1">
+      <c r="C20" s="184" t="s">
+        <v>13</v>
+      </c>
+      <c r="D20" s="185"/>
+      <c r="E20" s="185"/>
+      <c r="F20" s="185"/>
+      <c r="G20" s="185"/>
+      <c r="H20" s="40">
+        <f>SUM(H10:H19)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" ht="13.5" thickBot="1"/>
+    <row r="22" ht="18" customHeight="1" thickBot="1">
+      <c r="C22" s="186"/>
+      <c r="D22" s="187"/>
+      <c r="E22" s="187"/>
+      <c r="F22" s="187"/>
+      <c r="G22" s="187"/>
+      <c r="H22" s="188"/>
+    </row>
+    <row r="23" ht="15" customHeight="1">
+      <c r="C23" s="189" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" s="191" t="s">
+        <v>21</v>
+      </c>
+      <c r="E23" s="191" t="s">
+        <v>22</v>
+      </c>
+      <c r="F23" s="191" t="s">
+        <v>23</v>
+      </c>
+      <c r="G23" s="191" t="s">
+        <v>24</v>
+      </c>
+      <c r="H23" s="193" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="24" ht="13.9" customHeight="1" thickBot="1">
+      <c r="C24" s="190"/>
+      <c r="D24" s="192"/>
+      <c r="E24" s="192"/>
+      <c r="F24" s="192"/>
+      <c r="G24" s="192"/>
+      <c r="H24" s="194"/>
+    </row>
+    <row r="25" ht="14.5" customHeight="1">
+      <c r="C25" s="21"/>
+      <c r="D25" s="27"/>
+      <c r="E25" s="23"/>
+      <c r="F25" s="23"/>
+      <c r="G25" s="28"/>
+      <c r="H25" s="25"/>
+    </row>
+    <row r="26" ht="14.5" customHeight="1">
+      <c r="C26" s="21"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="23"/>
+      <c r="F26" s="23"/>
+      <c r="G26" s="28"/>
+      <c r="H26" s="25"/>
+    </row>
+    <row r="27" ht="14.5" customHeight="1">
+      <c r="C27" s="21"/>
+      <c r="D27" s="27"/>
+      <c r="E27" s="23"/>
+      <c r="F27" s="23"/>
+      <c r="G27" s="28"/>
+      <c r="H27" s="25"/>
+    </row>
+    <row r="28" ht="14.5" customHeight="1">
+      <c r="C28" s="21"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="23"/>
+      <c r="F28" s="23"/>
+      <c r="G28" s="28"/>
+      <c r="H28" s="25"/>
+    </row>
+    <row r="29" ht="14.5" customHeight="1">
+      <c r="C29" s="21"/>
+      <c r="D29" s="27"/>
+      <c r="E29" s="23"/>
+      <c r="F29" s="23"/>
+      <c r="G29" s="28"/>
+      <c r="H29" s="25"/>
+    </row>
+    <row r="30" ht="14.5" customHeight="1">
+      <c r="C30" s="21"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="23"/>
+      <c r="F30" s="23"/>
+      <c r="G30" s="28"/>
+      <c r="H30" s="25"/>
+    </row>
+    <row r="31" ht="14.5" customHeight="1">
+      <c r="C31" s="21"/>
+      <c r="D31" s="27"/>
+      <c r="E31" s="23"/>
+      <c r="F31" s="23"/>
+      <c r="G31" s="28"/>
+      <c r="H31" s="25"/>
+    </row>
+    <row r="32" ht="14.5" customHeight="1">
+      <c r="C32" s="21"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="23"/>
+      <c r="F32" s="23"/>
+      <c r="G32" s="28"/>
+      <c r="H32" s="25"/>
+    </row>
+    <row r="33" ht="14.5" customHeight="1">
+      <c r="C33" s="21"/>
+      <c r="D33" s="27"/>
+      <c r="E33" s="23"/>
+      <c r="F33" s="23"/>
+      <c r="G33" s="28"/>
+      <c r="H33" s="25"/>
+    </row>
+    <row r="34" ht="15" thickBot="1">
+      <c r="C34" s="34"/>
+      <c r="D34" s="35"/>
+      <c r="E34" s="36"/>
+      <c r="F34" s="36"/>
+      <c r="G34" s="38"/>
+      <c r="H34" s="39"/>
+    </row>
+    <row r="35" ht="16.5" thickBot="1">
+      <c r="C35" s="184" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" s="185"/>
+      <c r="E35" s="185"/>
+      <c r="F35" s="185"/>
+      <c r="G35" s="185"/>
+      <c r="H35" s="40">
+        <f>SUM(H25:H34)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" ht="13.5" thickBot="1">
+      <c r="H36" s="42"/>
+    </row>
+    <row r="37" ht="18" customHeight="1" thickBot="1">
+      <c r="C37" s="186"/>
+      <c r="D37" s="187"/>
+      <c r="E37" s="187"/>
+      <c r="F37" s="187"/>
+      <c r="G37" s="187"/>
+      <c r="H37" s="188"/>
+    </row>
+    <row r="38" ht="15" customHeight="1">
+      <c r="C38" s="189" t="s">
+        <v>20</v>
+      </c>
+      <c r="D38" s="191" t="s">
+        <v>21</v>
+      </c>
+      <c r="E38" s="191" t="s">
+        <v>22</v>
+      </c>
+      <c r="F38" s="191" t="s">
+        <v>23</v>
+      </c>
+      <c r="G38" s="191" t="s">
+        <v>24</v>
+      </c>
+      <c r="H38" s="193" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="39" ht="13.9" customHeight="1" thickBot="1">
+      <c r="C39" s="190"/>
+      <c r="D39" s="192"/>
+      <c r="E39" s="192"/>
+      <c r="F39" s="192"/>
+      <c r="G39" s="192"/>
+      <c r="H39" s="194"/>
+    </row>
+    <row r="40" ht="14.5" customHeight="1">
+      <c r="C40" s="21"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="23"/>
+      <c r="F40" s="23"/>
+      <c r="G40" s="28"/>
+      <c r="H40" s="25"/>
+    </row>
+    <row r="41" ht="14.5" customHeight="1">
+      <c r="C41" s="21"/>
+      <c r="D41" s="27"/>
+      <c r="E41" s="23"/>
+      <c r="F41" s="23"/>
+      <c r="G41" s="28"/>
+      <c r="H41" s="25"/>
+    </row>
+    <row r="42" ht="14.5" customHeight="1">
+      <c r="C42" s="21"/>
+      <c r="D42" s="27"/>
+      <c r="E42" s="23"/>
+      <c r="F42" s="23"/>
+      <c r="G42" s="28"/>
+      <c r="H42" s="25"/>
+    </row>
+    <row r="43" ht="14.5" customHeight="1">
+      <c r="C43" s="21"/>
+      <c r="D43" s="27"/>
+      <c r="E43" s="23"/>
+      <c r="F43" s="23"/>
+      <c r="G43" s="28"/>
+      <c r="H43" s="25"/>
+    </row>
+    <row r="44" ht="14.5" customHeight="1">
+      <c r="C44" s="21"/>
+      <c r="D44" s="27"/>
+      <c r="E44" s="23"/>
+      <c r="F44" s="23"/>
+      <c r="G44" s="28"/>
+      <c r="H44" s="25"/>
+    </row>
+    <row r="45" ht="14.5" customHeight="1">
+      <c r="C45" s="21"/>
+      <c r="D45" s="27"/>
+      <c r="E45" s="23"/>
+      <c r="F45" s="23"/>
+      <c r="G45" s="28"/>
+      <c r="H45" s="25"/>
+    </row>
+    <row r="46" ht="14.5" customHeight="1">
+      <c r="C46" s="21"/>
+      <c r="D46" s="27"/>
+      <c r="E46" s="23"/>
+      <c r="F46" s="23"/>
+      <c r="G46" s="28"/>
+      <c r="H46" s="25"/>
+    </row>
+    <row r="47" ht="14.5" customHeight="1">
+      <c r="C47" s="21"/>
+      <c r="D47" s="27"/>
+      <c r="E47" s="23"/>
+      <c r="F47" s="23"/>
+      <c r="G47" s="28"/>
+      <c r="H47" s="25"/>
+    </row>
+    <row r="48" ht="14.5" customHeight="1">
+      <c r="C48" s="21"/>
+      <c r="D48" s="27"/>
+      <c r="E48" s="23"/>
+      <c r="F48" s="23"/>
+      <c r="G48" s="28"/>
+      <c r="H48" s="25"/>
+    </row>
+    <row r="49" ht="15" thickBot="1">
+      <c r="C49" s="34"/>
+      <c r="D49" s="35"/>
+      <c r="E49" s="36"/>
+      <c r="F49" s="36"/>
+      <c r="G49" s="38"/>
+      <c r="H49" s="39"/>
+    </row>
+    <row r="50" ht="16.5" thickBot="1">
+      <c r="C50" s="184" t="s">
+        <v>13</v>
+      </c>
+      <c r="D50" s="185"/>
+      <c r="E50" s="185"/>
+      <c r="F50" s="185"/>
+      <c r="G50" s="185"/>
+      <c r="H50" s="40">
+        <f>SUM(H40:H49)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" ht="13.5" thickBot="1">
+      <c r="H51" s="43"/>
+    </row>
+    <row r="52" ht="18" customHeight="1" thickBot="1">
+      <c r="C52" s="186"/>
+      <c r="D52" s="187"/>
+      <c r="E52" s="187"/>
+      <c r="F52" s="187"/>
+      <c r="G52" s="187"/>
+      <c r="H52" s="188"/>
+    </row>
+    <row r="53" ht="15" customHeight="1">
+      <c r="C53" s="189" t="s">
+        <v>20</v>
+      </c>
+      <c r="D53" s="191" t="s">
+        <v>21</v>
+      </c>
+      <c r="E53" s="191" t="s">
+        <v>22</v>
+      </c>
+      <c r="F53" s="191" t="s">
+        <v>23</v>
+      </c>
+      <c r="G53" s="191" t="s">
+        <v>24</v>
+      </c>
+      <c r="H53" s="193" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="54" ht="13.9" customHeight="1" thickBot="1">
+      <c r="C54" s="190"/>
+      <c r="D54" s="192"/>
+      <c r="E54" s="192"/>
+      <c r="F54" s="192"/>
+      <c r="G54" s="192"/>
+      <c r="H54" s="194"/>
+    </row>
+    <row r="55" ht="14.5" customHeight="1">
+      <c r="C55" s="21"/>
+      <c r="D55" s="27"/>
+      <c r="E55" s="23"/>
+      <c r="F55" s="23"/>
+      <c r="G55" s="28"/>
+      <c r="H55" s="25"/>
+    </row>
+    <row r="56" ht="14.5" customHeight="1">
+      <c r="C56" s="21"/>
+      <c r="D56" s="27"/>
+      <c r="E56" s="23"/>
+      <c r="F56" s="23"/>
+      <c r="G56" s="28"/>
+      <c r="H56" s="25"/>
+    </row>
+    <row r="57" ht="14.5" customHeight="1">
+      <c r="C57" s="21"/>
+      <c r="D57" s="27"/>
+      <c r="E57" s="23"/>
+      <c r="F57" s="23"/>
+      <c r="G57" s="28"/>
+      <c r="H57" s="25"/>
+    </row>
+    <row r="58" ht="14.5" customHeight="1">
+      <c r="C58" s="21"/>
+      <c r="D58" s="27"/>
+      <c r="E58" s="23"/>
+      <c r="F58" s="23"/>
+      <c r="G58" s="28"/>
+      <c r="H58" s="25"/>
+    </row>
+    <row r="59" ht="14.5" customHeight="1">
+      <c r="C59" s="21"/>
+      <c r="D59" s="27"/>
+      <c r="E59" s="23"/>
+      <c r="F59" s="23"/>
+      <c r="G59" s="28"/>
+      <c r="H59" s="25"/>
+    </row>
+    <row r="60" ht="14.5" customHeight="1">
+      <c r="C60" s="21"/>
+      <c r="D60" s="27"/>
+      <c r="E60" s="23"/>
+      <c r="F60" s="23"/>
+      <c r="G60" s="28"/>
+      <c r="H60" s="25"/>
+    </row>
+    <row r="61" ht="14.5" customHeight="1">
+      <c r="C61" s="21"/>
+      <c r="D61" s="27"/>
+      <c r="E61" s="23"/>
+      <c r="F61" s="23"/>
+      <c r="G61" s="28"/>
+      <c r="H61" s="25"/>
+    </row>
+    <row r="62" ht="14.5" customHeight="1">
+      <c r="C62" s="21"/>
+      <c r="D62" s="27"/>
+      <c r="E62" s="23"/>
+      <c r="F62" s="23"/>
+      <c r="G62" s="28"/>
+      <c r="H62" s="25"/>
+    </row>
+    <row r="63" ht="14.5" customHeight="1">
+      <c r="C63" s="21"/>
+      <c r="D63" s="27"/>
+      <c r="E63" s="23"/>
+      <c r="F63" s="23"/>
+      <c r="G63" s="28"/>
+      <c r="H63" s="25"/>
+    </row>
+    <row r="64" ht="15" thickBot="1">
+      <c r="C64" s="34"/>
+      <c r="D64" s="35"/>
+      <c r="E64" s="36"/>
+      <c r="F64" s="36"/>
+      <c r="G64" s="38"/>
+      <c r="H64" s="39"/>
+    </row>
+    <row r="65" ht="16.5" thickBot="1">
+      <c r="C65" s="184" t="s">
+        <v>13</v>
+      </c>
+      <c r="D65" s="185"/>
+      <c r="E65" s="185"/>
+      <c r="F65" s="185"/>
+      <c r="G65" s="185"/>
+      <c r="H65" s="40">
+        <f>SUM(H55:H64)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" ht="6" customHeight="1"/>
+    <row r="67" ht="21.4" customHeight="1" thickBot="1">
+      <c r="C67" s="180" t="inlineStr">
+        <is>
+          <t>Grand Total</t>
+        </is>
+      </c>
+      <c r="D67" s="181"/>
+      <c r="E67" s="181"/>
+      <c r="F67" s="181"/>
+      <c r="G67" s="182"/>
+      <c r="H67" s="50"/>
+    </row>
+  </sheetData>
+  <mergeCells count="34">
+    <mergeCell ref="C2:H5"/>
+    <mergeCell ref="C7:H7"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="C20:G20"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="G23:G24"/>
+    <mergeCell ref="H23:H24"/>
+    <mergeCell ref="C35:G35"/>
+    <mergeCell ref="C37:H37"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:D39"/>
+    <mergeCell ref="E38:E39"/>
+    <mergeCell ref="F38:F39"/>
+    <mergeCell ref="G38:G39"/>
+    <mergeCell ref="H38:H39"/>
+    <mergeCell ref="C50:G50"/>
+    <mergeCell ref="C52:H52"/>
+    <mergeCell ref="C53:C54"/>
+    <mergeCell ref="D53:D54"/>
+    <mergeCell ref="E53:E54"/>
+    <mergeCell ref="F53:F54"/>
+    <mergeCell ref="G53:G54"/>
+    <mergeCell ref="H53:H54"/>
+    <mergeCell ref="C65:G65"/>
+    <mergeCell ref="C67:G67"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="90" fitToWidth="1" fitToHeight="0" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>

</xml_diff>